<commit_message>
Detect under-40 PIs whose name only is printed in green (LS6, SH5)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/prin_out/prin2026_funded_projects.xlsx
+++ b/prin_out/prin2026_funded_projects.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="All units" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All units" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All units'!$A$1:$J$752</definedName>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Università degli Studi "G. d'Annunzio" CHIETI-PESCARA</t>
+          <t>Università degli Studi "G. d'Annunzio" CHIETI- PESCARA</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">

</xml_diff>